<commit_message>
August 26th figure updates
</commit_message>
<xml_diff>
--- a/Sup Table 2 - annotations/Annotations_table_v2.xlsx
+++ b/Sup Table 2 - annotations/Annotations_table_v2.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30224"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Labs\Farber_Lab\Farber_Lab_Public\snRNA-seq\atlas paper figures\Sup Table 2 - annotations\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://livejohnshopkins-my.sharepoint.com/personal/cbrow222_jh_edu/Documents/Farber_Lab/Atlas paper/Brown_Biederman_et_al_2026_code_and_figures/Sup Table 2 - annotations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{4ED11F6D-2052-45AB-9608-AE983135E3D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9807CB37-2F42-4CA8-AB9C-853A063CEEA6}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{4ED11F6D-2052-45AB-9608-AE983135E3D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C35D95BB-74D0-4836-A30B-A25B3BBF81D0}"/>
   <bookViews>
-    <workbookView xWindow="-29910" yWindow="2670" windowWidth="22845" windowHeight="15855" xr2:uid="{FF2C5148-4215-4530-974F-5E7313BCF37D}"/>
+    <workbookView xWindow="-32535" yWindow="540" windowWidth="32370" windowHeight="19500" xr2:uid="{FF2C5148-4215-4530-974F-5E7313BCF37D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$2:$J$273</definedName>
+  </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -4254,7 +4257,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4620,26 +4623,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56E4E094-9D27-4105-A489-8372C22533B2}">
   <dimension ref="A1:J273"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="65.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="61.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="67.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="65.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="61.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="67.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="27.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -4671,7 +4674,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>195</v>
       </c>
@@ -4703,7 +4706,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>46</v>
       </c>
@@ -4735,7 +4738,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>60</v>
       </c>
@@ -4767,7 +4770,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>189</v>
       </c>
@@ -4799,7 +4802,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>158</v>
       </c>
@@ -4831,7 +4834,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>238</v>
       </c>
@@ -4863,7 +4866,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>163</v>
       </c>
@@ -4895,7 +4898,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>79</v>
       </c>
@@ -4927,7 +4930,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>261</v>
       </c>
@@ -4959,7 +4962,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>113</v>
       </c>
@@ -4991,7 +4994,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>69</v>
       </c>
@@ -5023,7 +5026,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>214</v>
       </c>
@@ -5055,7 +5058,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>59</v>
       </c>
@@ -5087,7 +5090,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>177</v>
       </c>
@@ -5119,7 +5122,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="17" spans="1:10">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>145</v>
       </c>
@@ -5151,7 +5154,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="18" spans="1:10">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>142</v>
       </c>
@@ -5183,7 +5186,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="19" spans="1:10">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>257</v>
       </c>
@@ -5215,7 +5218,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="20" spans="1:10">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>114</v>
       </c>
@@ -5247,7 +5250,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="21" spans="1:10">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>129</v>
       </c>
@@ -5279,7 +5282,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="22" spans="1:10">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>128</v>
       </c>
@@ -5311,7 +5314,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="23" spans="1:10">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>95</v>
       </c>
@@ -5343,7 +5346,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="24" spans="1:10">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>33</v>
       </c>
@@ -5375,7 +5378,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="25" spans="1:10">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>32</v>
       </c>
@@ -5407,7 +5410,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="26" spans="1:10">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>37</v>
       </c>
@@ -5439,7 +5442,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="27" spans="1:10">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>27</v>
       </c>
@@ -5471,7 +5474,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="28" spans="1:10">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>4</v>
       </c>
@@ -5503,7 +5506,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="29" spans="1:10">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>127</v>
       </c>
@@ -5535,7 +5538,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="30" spans="1:10">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>38</v>
       </c>
@@ -5567,7 +5570,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="31" spans="1:10">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>36</v>
       </c>
@@ -5599,7 +5602,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="32" spans="1:10">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -5631,7 +5634,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="33" spans="1:10">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>226</v>
       </c>
@@ -5663,7 +5666,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="34" spans="1:10">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>260</v>
       </c>
@@ -5695,7 +5698,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="35" spans="1:10">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>72</v>
       </c>
@@ -5727,7 +5730,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="36" spans="1:10">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>34</v>
       </c>
@@ -5759,7 +5762,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="37" spans="1:10">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>56</v>
       </c>
@@ -5791,7 +5794,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="38" spans="1:10">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>74</v>
       </c>
@@ -5823,7 +5826,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="39" spans="1:10">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>11</v>
       </c>
@@ -5855,7 +5858,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="40" spans="1:10">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>237</v>
       </c>
@@ -5887,7 +5890,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="41" spans="1:10">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>255</v>
       </c>
@@ -5919,7 +5922,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="42" spans="1:10">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>253</v>
       </c>
@@ -5951,7 +5954,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="43" spans="1:10">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>153</v>
       </c>
@@ -5983,7 +5986,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="44" spans="1:10">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>64</v>
       </c>
@@ -6015,7 +6018,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="45" spans="1:10">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>132</v>
       </c>
@@ -6047,7 +6050,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="46" spans="1:10">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>176</v>
       </c>
@@ -6079,7 +6082,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="47" spans="1:10">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>94</v>
       </c>
@@ -6111,7 +6114,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="48" spans="1:10">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>208</v>
       </c>
@@ -6143,7 +6146,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="49" spans="1:10">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>112</v>
       </c>
@@ -6175,7 +6178,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="50" spans="1:10">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>186</v>
       </c>
@@ -6207,7 +6210,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="51" spans="1:10">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>216</v>
       </c>
@@ -6239,7 +6242,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="52" spans="1:10">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>171</v>
       </c>
@@ -6271,7 +6274,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="53" spans="1:10">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>232</v>
       </c>
@@ -6303,7 +6306,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="54" spans="1:10">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>151</v>
       </c>
@@ -6335,7 +6338,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="55" spans="1:10">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>156</v>
       </c>
@@ -6367,7 +6370,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="56" spans="1:10">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>39</v>
       </c>
@@ -6399,7 +6402,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="57" spans="1:10">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>188</v>
       </c>
@@ -6431,7 +6434,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="58" spans="1:10">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>118</v>
       </c>
@@ -6463,7 +6466,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="59" spans="1:10">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>26</v>
       </c>
@@ -6495,7 +6498,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="60" spans="1:10">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>97</v>
       </c>
@@ -6527,7 +6530,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="61" spans="1:10">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>103</v>
       </c>
@@ -6559,7 +6562,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="62" spans="1:10">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>41</v>
       </c>
@@ -6591,7 +6594,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="63" spans="1:10">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>49</v>
       </c>
@@ -6623,7 +6626,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="64" spans="1:10">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>235</v>
       </c>
@@ -6655,7 +6658,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="65" spans="1:10">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>233</v>
       </c>
@@ -6687,7 +6690,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="66" spans="1:10">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>106</v>
       </c>
@@ -6719,7 +6722,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="67" spans="1:10">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>126</v>
       </c>
@@ -6751,7 +6754,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="68" spans="1:10">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>229</v>
       </c>
@@ -6783,7 +6786,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="69" spans="1:10">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>123</v>
       </c>
@@ -6815,7 +6818,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="70" spans="1:10">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>207</v>
       </c>
@@ -6847,7 +6850,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="71" spans="1:10">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>225</v>
       </c>
@@ -6879,7 +6882,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="72" spans="1:10">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>174</v>
       </c>
@@ -6911,7 +6914,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="73" spans="1:10">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>68</v>
       </c>
@@ -6943,7 +6946,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="74" spans="1:10">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>28</v>
       </c>
@@ -6975,7 +6978,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="75" spans="1:10">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>99</v>
       </c>
@@ -7007,7 +7010,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="76" spans="1:10">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>44</v>
       </c>
@@ -7039,7 +7042,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="77" spans="1:10">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>252</v>
       </c>
@@ -7071,7 +7074,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="78" spans="1:10">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>105</v>
       </c>
@@ -7103,7 +7106,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="79" spans="1:10">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>42</v>
       </c>
@@ -7135,7 +7138,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="80" spans="1:10">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>119</v>
       </c>
@@ -7167,7 +7170,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="81" spans="1:10">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>24</v>
       </c>
@@ -7199,7 +7202,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="82" spans="1:10">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>21</v>
       </c>
@@ -7231,7 +7234,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="83" spans="1:10">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>35</v>
       </c>
@@ -7263,7 +7266,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="84" spans="1:10">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>187</v>
       </c>
@@ -7295,7 +7298,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="85" spans="1:10">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>14</v>
       </c>
@@ -7327,7 +7330,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="86" spans="1:10">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>191</v>
       </c>
@@ -7359,7 +7362,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="87" spans="1:10">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>22</v>
       </c>
@@ -7391,7 +7394,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="88" spans="1:10">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>213</v>
       </c>
@@ -7423,7 +7426,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="89" spans="1:10">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>152</v>
       </c>
@@ -7455,7 +7458,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="90" spans="1:10">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>204</v>
       </c>
@@ -7487,7 +7490,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="91" spans="1:10">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>160</v>
       </c>
@@ -7519,7 +7522,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="92" spans="1:10">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>51</v>
       </c>
@@ -7551,7 +7554,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="93" spans="1:10">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>30</v>
       </c>
@@ -7583,7 +7586,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="94" spans="1:10">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>157</v>
       </c>
@@ -7615,7 +7618,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="95" spans="1:10">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>65</v>
       </c>
@@ -7647,7 +7650,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="96" spans="1:10">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>211</v>
       </c>
@@ -7679,7 +7682,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="97" spans="1:10">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>166</v>
       </c>
@@ -7711,7 +7714,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="98" spans="1:10">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>242</v>
       </c>
@@ -7743,7 +7746,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="99" spans="1:10">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>202</v>
       </c>
@@ -7775,7 +7778,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="100" spans="1:10">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>179</v>
       </c>
@@ -7807,7 +7810,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="101" spans="1:10">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>215</v>
       </c>
@@ -7839,7 +7842,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="102" spans="1:10">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>140</v>
       </c>
@@ -7871,7 +7874,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="103" spans="1:10">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>256</v>
       </c>
@@ -7903,7 +7906,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="104" spans="1:10">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>77</v>
       </c>
@@ -7935,7 +7938,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="105" spans="1:10">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>264</v>
       </c>
@@ -7967,7 +7970,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="106" spans="1:10">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>162</v>
       </c>
@@ -7999,7 +8002,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="107" spans="1:10">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>141</v>
       </c>
@@ -8031,7 +8034,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="108" spans="1:10">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>250</v>
       </c>
@@ -8063,7 +8066,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="109" spans="1:10">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>246</v>
       </c>
@@ -8095,7 +8098,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="110" spans="1:10">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>266</v>
       </c>
@@ -8127,7 +8130,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="111" spans="1:10">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>175</v>
       </c>
@@ -8159,7 +8162,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="112" spans="1:10">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>43</v>
       </c>
@@ -8191,7 +8194,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="113" spans="1:10">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>220</v>
       </c>
@@ -8223,7 +8226,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="114" spans="1:10">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>164</v>
       </c>
@@ -8255,7 +8258,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="115" spans="1:10">
+    <row r="115" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>149</v>
       </c>
@@ -8287,7 +8290,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="116" spans="1:10">
+    <row r="116" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>78</v>
       </c>
@@ -8319,7 +8322,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="117" spans="1:10">
+    <row r="117" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>62</v>
       </c>
@@ -8351,7 +8354,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="118" spans="1:10">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>55</v>
       </c>
@@ -8383,7 +8386,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="119" spans="1:10">
+    <row r="119" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>89</v>
       </c>
@@ -8415,7 +8418,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="120" spans="1:10">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>115</v>
       </c>
@@ -8447,7 +8450,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="121" spans="1:10">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>104</v>
       </c>
@@ -8479,7 +8482,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="122" spans="1:10">
+    <row r="122" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>45</v>
       </c>
@@ -8511,7 +8514,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="123" spans="1:10">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>183</v>
       </c>
@@ -8543,7 +8546,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="124" spans="1:10">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>148</v>
       </c>
@@ -8575,7 +8578,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="125" spans="1:10">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>263</v>
       </c>
@@ -8607,7 +8610,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="126" spans="1:10">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>102</v>
       </c>
@@ -8639,7 +8642,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="127" spans="1:10">
+    <row r="127" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>91</v>
       </c>
@@ -8671,7 +8674,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="128" spans="1:10">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>131</v>
       </c>
@@ -8703,7 +8706,7 @@
         <v>705</v>
       </c>
     </row>
-    <row r="129" spans="1:10">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>193</v>
       </c>
@@ -8735,7 +8738,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="130" spans="1:10">
+    <row r="130" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>227</v>
       </c>
@@ -8767,7 +8770,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="131" spans="1:10">
+    <row r="131" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>190</v>
       </c>
@@ -8799,7 +8802,7 @@
         <v>721</v>
       </c>
     </row>
-    <row r="132" spans="1:10">
+    <row r="132" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>159</v>
       </c>
@@ -8831,7 +8834,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="133" spans="1:10">
+    <row r="133" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>144</v>
       </c>
@@ -8863,7 +8866,7 @@
         <v>731</v>
       </c>
     </row>
-    <row r="134" spans="1:10">
+    <row r="134" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>196</v>
       </c>
@@ -8895,7 +8898,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="135" spans="1:10">
+    <row r="135" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>133</v>
       </c>
@@ -8927,7 +8930,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="136" spans="1:10">
+    <row r="136" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>236</v>
       </c>
@@ -8959,7 +8962,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="137" spans="1:10">
+    <row r="137" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>107</v>
       </c>
@@ -8991,7 +8994,7 @@
         <v>746</v>
       </c>
     </row>
-    <row r="138" spans="1:10">
+    <row r="138" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>199</v>
       </c>
@@ -9023,7 +9026,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="139" spans="1:10">
+    <row r="139" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>87</v>
       </c>
@@ -9055,7 +9058,7 @@
         <v>754</v>
       </c>
     </row>
-    <row r="140" spans="1:10">
+    <row r="140" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>210</v>
       </c>
@@ -9087,7 +9090,7 @@
         <v>758</v>
       </c>
     </row>
-    <row r="141" spans="1:10">
+    <row r="141" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>178</v>
       </c>
@@ -9119,7 +9122,7 @@
         <v>762</v>
       </c>
     </row>
-    <row r="142" spans="1:10">
+    <row r="142" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>138</v>
       </c>
@@ -9151,7 +9154,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="143" spans="1:10">
+    <row r="143" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>170</v>
       </c>
@@ -9183,7 +9186,7 @@
         <v>770</v>
       </c>
     </row>
-    <row r="144" spans="1:10">
+    <row r="144" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>110</v>
       </c>
@@ -9215,7 +9218,7 @@
         <v>773</v>
       </c>
     </row>
-    <row r="145" spans="1:10">
+    <row r="145" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A145">
         <v>83</v>
       </c>
@@ -9247,7 +9250,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="146" spans="1:10">
+    <row r="146" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A146">
         <v>76</v>
       </c>
@@ -9279,7 +9282,7 @@
         <v>779</v>
       </c>
     </row>
-    <row r="147" spans="1:10">
+    <row r="147" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>54</v>
       </c>
@@ -9311,7 +9314,7 @@
         <v>783</v>
       </c>
     </row>
-    <row r="148" spans="1:10">
+    <row r="148" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>201</v>
       </c>
@@ -9343,7 +9346,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="149" spans="1:10">
+    <row r="149" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>117</v>
       </c>
@@ -9375,7 +9378,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="150" spans="1:10">
+    <row r="150" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>249</v>
       </c>
@@ -9407,7 +9410,7 @@
         <v>797</v>
       </c>
     </row>
-    <row r="151" spans="1:10">
+    <row r="151" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>137</v>
       </c>
@@ -9439,7 +9442,7 @@
         <v>803</v>
       </c>
     </row>
-    <row r="152" spans="1:10">
+    <row r="152" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>245</v>
       </c>
@@ -9471,7 +9474,7 @@
         <v>809</v>
       </c>
     </row>
-    <row r="153" spans="1:10">
+    <row r="153" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>218</v>
       </c>
@@ -9503,7 +9506,7 @@
         <v>815</v>
       </c>
     </row>
-    <row r="154" spans="1:10">
+    <row r="154" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>125</v>
       </c>
@@ -9535,7 +9538,7 @@
         <v>821</v>
       </c>
     </row>
-    <row r="155" spans="1:10">
+    <row r="155" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>147</v>
       </c>
@@ -9567,7 +9570,7 @@
         <v>827</v>
       </c>
     </row>
-    <row r="156" spans="1:10">
+    <row r="156" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>8</v>
       </c>
@@ -9599,7 +9602,7 @@
         <v>831</v>
       </c>
     </row>
-    <row r="157" spans="1:10">
+    <row r="157" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>209</v>
       </c>
@@ -9631,7 +9634,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="158" spans="1:10">
+    <row r="158" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>7</v>
       </c>
@@ -9663,7 +9666,7 @@
         <v>841</v>
       </c>
     </row>
-    <row r="159" spans="1:10">
+    <row r="159" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>3</v>
       </c>
@@ -9695,7 +9698,7 @@
         <v>848</v>
       </c>
     </row>
-    <row r="160" spans="1:10">
+    <row r="160" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>0</v>
       </c>
@@ -9727,7 +9730,7 @@
         <v>852</v>
       </c>
     </row>
-    <row r="161" spans="1:10">
+    <row r="161" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A161">
         <v>15</v>
       </c>
@@ -9759,7 +9762,7 @@
         <v>858</v>
       </c>
     </row>
-    <row r="162" spans="1:10">
+    <row r="162" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>101</v>
       </c>
@@ -9791,7 +9794,7 @@
         <v>862</v>
       </c>
     </row>
-    <row r="163" spans="1:10">
+    <row r="163" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>29</v>
       </c>
@@ -9823,7 +9826,7 @@
         <v>866</v>
       </c>
     </row>
-    <row r="164" spans="1:10">
+    <row r="164" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A164">
         <v>173</v>
       </c>
@@ -9855,7 +9858,7 @@
         <v>872</v>
       </c>
     </row>
-    <row r="165" spans="1:10">
+    <row r="165" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A165">
         <v>243</v>
       </c>
@@ -9887,7 +9890,7 @@
         <v>876</v>
       </c>
     </row>
-    <row r="166" spans="1:10">
+    <row r="166" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A166">
         <v>192</v>
       </c>
@@ -9919,7 +9922,7 @@
         <v>880</v>
       </c>
     </row>
-    <row r="167" spans="1:10">
+    <row r="167" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A167">
         <v>80</v>
       </c>
@@ -9951,7 +9954,7 @@
         <v>886</v>
       </c>
     </row>
-    <row r="168" spans="1:10">
+    <row r="168" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A168">
         <v>198</v>
       </c>
@@ -9983,7 +9986,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="169" spans="1:10">
+    <row r="169" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A169">
         <v>124</v>
       </c>
@@ -10015,7 +10018,7 @@
         <v>898</v>
       </c>
     </row>
-    <row r="170" spans="1:10">
+    <row r="170" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A170">
         <v>53</v>
       </c>
@@ -10047,7 +10050,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="171" spans="1:10">
+    <row r="171" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A171">
         <v>2</v>
       </c>
@@ -10079,7 +10082,7 @@
         <v>906</v>
       </c>
     </row>
-    <row r="172" spans="1:10">
+    <row r="172" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A172">
         <v>120</v>
       </c>
@@ -10111,7 +10114,7 @@
         <v>910</v>
       </c>
     </row>
-    <row r="173" spans="1:10">
+    <row r="173" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A173">
         <v>239</v>
       </c>
@@ -10143,7 +10146,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="174" spans="1:10">
+    <row r="174" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>219</v>
       </c>
@@ -10175,7 +10178,7 @@
         <v>920</v>
       </c>
     </row>
-    <row r="175" spans="1:10">
+    <row r="175" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A175">
         <v>181</v>
       </c>
@@ -10207,7 +10210,7 @@
         <v>926</v>
       </c>
     </row>
-    <row r="176" spans="1:10">
+    <row r="176" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A176">
         <v>267</v>
       </c>
@@ -10239,7 +10242,7 @@
         <v>932</v>
       </c>
     </row>
-    <row r="177" spans="1:10">
+    <row r="177" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>262</v>
       </c>
@@ -10271,7 +10274,7 @@
         <v>936</v>
       </c>
     </row>
-    <row r="178" spans="1:10">
+    <row r="178" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>185</v>
       </c>
@@ -10303,7 +10306,7 @@
         <v>942</v>
       </c>
     </row>
-    <row r="179" spans="1:10">
+    <row r="179" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>169</v>
       </c>
@@ -10335,7 +10338,7 @@
         <v>946</v>
       </c>
     </row>
-    <row r="180" spans="1:10">
+    <row r="180" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A180">
         <v>150</v>
       </c>
@@ -10367,7 +10370,7 @@
         <v>950</v>
       </c>
     </row>
-    <row r="181" spans="1:10">
+    <row r="181" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A181">
         <v>241</v>
       </c>
@@ -10399,7 +10402,7 @@
         <v>956</v>
       </c>
     </row>
-    <row r="182" spans="1:10">
+    <row r="182" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A182">
         <v>212</v>
       </c>
@@ -10431,7 +10434,7 @@
         <v>962</v>
       </c>
     </row>
-    <row r="183" spans="1:10">
+    <row r="183" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A183">
         <v>194</v>
       </c>
@@ -10463,7 +10466,7 @@
         <v>968</v>
       </c>
     </row>
-    <row r="184" spans="1:10">
+    <row r="184" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A184">
         <v>269</v>
       </c>
@@ -10495,7 +10498,7 @@
         <v>972</v>
       </c>
     </row>
-    <row r="185" spans="1:10">
+    <row r="185" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A185">
         <v>265</v>
       </c>
@@ -10527,7 +10530,7 @@
         <v>976</v>
       </c>
     </row>
-    <row r="186" spans="1:10">
+    <row r="186" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A186">
         <v>251</v>
       </c>
@@ -10559,7 +10562,7 @@
         <v>982</v>
       </c>
     </row>
-    <row r="187" spans="1:10">
+    <row r="187" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A187">
         <v>203</v>
       </c>
@@ -10591,7 +10594,7 @@
         <v>988</v>
       </c>
     </row>
-    <row r="188" spans="1:10">
+    <row r="188" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A188">
         <v>168</v>
       </c>
@@ -10623,7 +10626,7 @@
         <v>994</v>
       </c>
     </row>
-    <row r="189" spans="1:10">
+    <row r="189" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A189">
         <v>96</v>
       </c>
@@ -10655,7 +10658,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="190" spans="1:10">
+    <row r="190" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A190">
         <v>200</v>
       </c>
@@ -10687,7 +10690,7 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="191" spans="1:10">
+    <row r="191" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A191">
         <v>231</v>
       </c>
@@ -10719,7 +10722,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="192" spans="1:10">
+    <row r="192" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A192">
         <v>139</v>
       </c>
@@ -10751,7 +10754,7 @@
         <v>1018</v>
       </c>
     </row>
-    <row r="193" spans="1:10">
+    <row r="193" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A193">
         <v>223</v>
       </c>
@@ -10783,7 +10786,7 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="194" spans="1:10">
+    <row r="194" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A194">
         <v>182</v>
       </c>
@@ -10815,7 +10818,7 @@
         <v>1028</v>
       </c>
     </row>
-    <row r="195" spans="1:10">
+    <row r="195" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>270</v>
       </c>
@@ -10847,7 +10850,7 @@
         <v>1034</v>
       </c>
     </row>
-    <row r="196" spans="1:10">
+    <row r="196" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A196">
         <v>155</v>
       </c>
@@ -10879,7 +10882,7 @@
         <v>1040</v>
       </c>
     </row>
-    <row r="197" spans="1:10">
+    <row r="197" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A197">
         <v>143</v>
       </c>
@@ -10911,7 +10914,7 @@
         <v>1046</v>
       </c>
     </row>
-    <row r="198" spans="1:10">
+    <row r="198" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A198">
         <v>165</v>
       </c>
@@ -10943,7 +10946,7 @@
         <v>1052</v>
       </c>
     </row>
-    <row r="199" spans="1:10">
+    <row r="199" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A199">
         <v>172</v>
       </c>
@@ -10975,7 +10978,7 @@
         <v>1058</v>
       </c>
     </row>
-    <row r="200" spans="1:10">
+    <row r="200" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A200">
         <v>108</v>
       </c>
@@ -11007,7 +11010,7 @@
         <v>1062</v>
       </c>
     </row>
-    <row r="201" spans="1:10">
+    <row r="201" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A201">
         <v>224</v>
       </c>
@@ -11039,7 +11042,7 @@
         <v>1066</v>
       </c>
     </row>
-    <row r="202" spans="1:10">
+    <row r="202" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A202">
         <v>222</v>
       </c>
@@ -11071,7 +11074,7 @@
         <v>1070</v>
       </c>
     </row>
-    <row r="203" spans="1:10">
+    <row r="203" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A203">
         <v>258</v>
       </c>
@@ -11103,7 +11106,7 @@
         <v>1074</v>
       </c>
     </row>
-    <row r="204" spans="1:10">
+    <row r="204" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A204">
         <v>247</v>
       </c>
@@ -11135,7 +11138,7 @@
         <v>1081</v>
       </c>
     </row>
-    <row r="205" spans="1:10">
+    <row r="205" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A205">
         <v>154</v>
       </c>
@@ -11167,7 +11170,7 @@
         <v>1087</v>
       </c>
     </row>
-    <row r="206" spans="1:10">
+    <row r="206" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A206">
         <v>50</v>
       </c>
@@ -11199,7 +11202,7 @@
         <v>1093</v>
       </c>
     </row>
-    <row r="207" spans="1:10">
+    <row r="207" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A207">
         <v>254</v>
       </c>
@@ -11231,7 +11234,7 @@
         <v>1099</v>
       </c>
     </row>
-    <row r="208" spans="1:10">
+    <row r="208" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A208">
         <v>63</v>
       </c>
@@ -11263,7 +11266,7 @@
         <v>1103</v>
       </c>
     </row>
-    <row r="209" spans="1:10">
+    <row r="209" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A209">
         <v>23</v>
       </c>
@@ -11295,7 +11298,7 @@
         <v>1107</v>
       </c>
     </row>
-    <row r="210" spans="1:10">
+    <row r="210" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A210">
         <v>16</v>
       </c>
@@ -11327,7 +11330,7 @@
         <v>1111</v>
       </c>
     </row>
-    <row r="211" spans="1:10">
+    <row r="211" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A211">
         <v>206</v>
       </c>
@@ -11359,7 +11362,7 @@
         <v>1115</v>
       </c>
     </row>
-    <row r="212" spans="1:10">
+    <row r="212" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A212">
         <v>71</v>
       </c>
@@ -11391,7 +11394,7 @@
         <v>1119</v>
       </c>
     </row>
-    <row r="213" spans="1:10">
+    <row r="213" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A213">
         <v>130</v>
       </c>
@@ -11423,7 +11426,7 @@
         <v>1123</v>
       </c>
     </row>
-    <row r="214" spans="1:10">
+    <row r="214" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A214">
         <v>18</v>
       </c>
@@ -11455,7 +11458,7 @@
         <v>1129</v>
       </c>
     </row>
-    <row r="215" spans="1:10">
+    <row r="215" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A215">
         <v>5</v>
       </c>
@@ -11487,7 +11490,7 @@
         <v>1135</v>
       </c>
     </row>
-    <row r="216" spans="1:10">
+    <row r="216" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A216">
         <v>197</v>
       </c>
@@ -11519,7 +11522,7 @@
         <v>1141</v>
       </c>
     </row>
-    <row r="217" spans="1:10">
+    <row r="217" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A217">
         <v>259</v>
       </c>
@@ -11551,7 +11554,7 @@
         <v>1143</v>
       </c>
     </row>
-    <row r="218" spans="1:10">
+    <row r="218" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A218">
         <v>75</v>
       </c>
@@ -11583,7 +11586,7 @@
         <v>1147</v>
       </c>
     </row>
-    <row r="219" spans="1:10">
+    <row r="219" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A219">
         <v>240</v>
       </c>
@@ -11615,7 +11618,7 @@
         <v>1153</v>
       </c>
     </row>
-    <row r="220" spans="1:10">
+    <row r="220" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A220">
         <v>86</v>
       </c>
@@ -11647,7 +11650,7 @@
         <v>1156</v>
       </c>
     </row>
-    <row r="221" spans="1:10">
+    <row r="221" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A221">
         <v>230</v>
       </c>
@@ -11679,7 +11682,7 @@
         <v>1162</v>
       </c>
     </row>
-    <row r="222" spans="1:10">
+    <row r="222" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A222">
         <v>17</v>
       </c>
@@ -11711,7 +11714,7 @@
         <v>1168</v>
       </c>
     </row>
-    <row r="223" spans="1:10">
+    <row r="223" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A223">
         <v>58</v>
       </c>
@@ -11743,7 +11746,7 @@
         <v>1174</v>
       </c>
     </row>
-    <row r="224" spans="1:10">
+    <row r="224" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A224">
         <v>10</v>
       </c>
@@ -11775,7 +11778,7 @@
         <v>1178</v>
       </c>
     </row>
-    <row r="225" spans="1:10">
+    <row r="225" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A225">
         <v>57</v>
       </c>
@@ -11807,7 +11810,7 @@
         <v>1181</v>
       </c>
     </row>
-    <row r="226" spans="1:10">
+    <row r="226" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A226">
         <v>85</v>
       </c>
@@ -11839,7 +11842,7 @@
         <v>1187</v>
       </c>
     </row>
-    <row r="227" spans="1:10">
+    <row r="227" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A227">
         <v>217</v>
       </c>
@@ -11871,7 +11874,7 @@
         <v>1193</v>
       </c>
     </row>
-    <row r="228" spans="1:10">
+    <row r="228" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A228">
         <v>66</v>
       </c>
@@ -11903,7 +11906,7 @@
         <v>1199</v>
       </c>
     </row>
-    <row r="229" spans="1:10">
+    <row r="229" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A229">
         <v>92</v>
       </c>
@@ -11935,7 +11938,7 @@
         <v>1203</v>
       </c>
     </row>
-    <row r="230" spans="1:10">
+    <row r="230" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A230">
         <v>70</v>
       </c>
@@ -11967,7 +11970,7 @@
         <v>1209</v>
       </c>
     </row>
-    <row r="231" spans="1:10">
+    <row r="231" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A231">
         <v>13</v>
       </c>
@@ -11999,7 +12002,7 @@
         <v>1215</v>
       </c>
     </row>
-    <row r="232" spans="1:10">
+    <row r="232" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A232">
         <v>47</v>
       </c>
@@ -12031,7 +12034,7 @@
         <v>1221</v>
       </c>
     </row>
-    <row r="233" spans="1:10">
+    <row r="233" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A233">
         <v>228</v>
       </c>
@@ -12063,7 +12066,7 @@
         <v>1225</v>
       </c>
     </row>
-    <row r="234" spans="1:10">
+    <row r="234" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A234">
         <v>116</v>
       </c>
@@ -12095,7 +12098,7 @@
         <v>1231</v>
       </c>
     </row>
-    <row r="235" spans="1:10">
+    <row r="235" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A235">
         <v>40</v>
       </c>
@@ -12127,7 +12130,7 @@
         <v>1237</v>
       </c>
     </row>
-    <row r="236" spans="1:10">
+    <row r="236" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A236">
         <v>98</v>
       </c>
@@ -12159,7 +12162,7 @@
         <v>1241</v>
       </c>
     </row>
-    <row r="237" spans="1:10">
+    <row r="237" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A237">
         <v>100</v>
       </c>
@@ -12191,7 +12194,7 @@
         <v>1243</v>
       </c>
     </row>
-    <row r="238" spans="1:10">
+    <row r="238" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A238">
         <v>221</v>
       </c>
@@ -12223,7 +12226,7 @@
         <v>1249</v>
       </c>
     </row>
-    <row r="239" spans="1:10">
+    <row r="239" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A239">
         <v>248</v>
       </c>
@@ -12255,7 +12258,7 @@
         <v>1255</v>
       </c>
     </row>
-    <row r="240" spans="1:10">
+    <row r="240" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A240">
         <v>9</v>
       </c>
@@ -12287,7 +12290,7 @@
         <v>1261</v>
       </c>
     </row>
-    <row r="241" spans="1:10">
+    <row r="241" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A241">
         <v>6</v>
       </c>
@@ -12319,7 +12322,7 @@
         <v>1267</v>
       </c>
     </row>
-    <row r="242" spans="1:10">
+    <row r="242" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A242">
         <v>19</v>
       </c>
@@ -12351,7 +12354,7 @@
         <v>1273</v>
       </c>
     </row>
-    <row r="243" spans="1:10">
+    <row r="243" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A243">
         <v>109</v>
       </c>
@@ -12383,7 +12386,7 @@
         <v>1277</v>
       </c>
     </row>
-    <row r="244" spans="1:10">
+    <row r="244" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A244">
         <v>12</v>
       </c>
@@ -12415,7 +12418,7 @@
         <v>1281</v>
       </c>
     </row>
-    <row r="245" spans="1:10">
+    <row r="245" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A245">
         <v>48</v>
       </c>
@@ -12447,7 +12450,7 @@
         <v>1285</v>
       </c>
     </row>
-    <row r="246" spans="1:10">
+    <row r="246" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A246">
         <v>134</v>
       </c>
@@ -12479,7 +12482,7 @@
         <v>1287</v>
       </c>
     </row>
-    <row r="247" spans="1:10">
+    <row r="247" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A247">
         <v>180</v>
       </c>
@@ -12511,7 +12514,7 @@
         <v>1289</v>
       </c>
     </row>
-    <row r="248" spans="1:10">
+    <row r="248" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A248">
         <v>136</v>
       </c>
@@ -12543,7 +12546,7 @@
         <v>1295</v>
       </c>
     </row>
-    <row r="249" spans="1:10">
+    <row r="249" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A249">
         <v>161</v>
       </c>
@@ -12575,7 +12578,7 @@
         <v>1301</v>
       </c>
     </row>
-    <row r="250" spans="1:10">
+    <row r="250" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A250">
         <v>244</v>
       </c>
@@ -12607,7 +12610,7 @@
         <v>1307</v>
       </c>
     </row>
-    <row r="251" spans="1:10">
+    <row r="251" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A251">
         <v>205</v>
       </c>
@@ -12639,7 +12642,7 @@
         <v>1313</v>
       </c>
     </row>
-    <row r="252" spans="1:10">
+    <row r="252" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A252">
         <v>122</v>
       </c>
@@ -12671,7 +12674,7 @@
         <v>1319</v>
       </c>
     </row>
-    <row r="253" spans="1:10">
+    <row r="253" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A253">
         <v>90</v>
       </c>
@@ -12703,7 +12706,7 @@
         <v>1325</v>
       </c>
     </row>
-    <row r="254" spans="1:10">
+    <row r="254" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A254">
         <v>184</v>
       </c>
@@ -12735,7 +12738,7 @@
         <v>1329</v>
       </c>
     </row>
-    <row r="255" spans="1:10">
+    <row r="255" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A255">
         <v>121</v>
       </c>
@@ -12767,7 +12770,7 @@
         <v>1335</v>
       </c>
     </row>
-    <row r="256" spans="1:10">
+    <row r="256" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A256">
         <v>52</v>
       </c>
@@ -12799,7 +12802,7 @@
         <v>1339</v>
       </c>
     </row>
-    <row r="257" spans="1:10">
+    <row r="257" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A257">
         <v>1</v>
       </c>
@@ -12831,7 +12834,7 @@
         <v>1343</v>
       </c>
     </row>
-    <row r="258" spans="1:10">
+    <row r="258" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A258">
         <v>146</v>
       </c>
@@ -12863,7 +12866,7 @@
         <v>1349</v>
       </c>
     </row>
-    <row r="259" spans="1:10">
+    <row r="259" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A259">
         <v>73</v>
       </c>
@@ -12895,7 +12898,7 @@
         <v>1353</v>
       </c>
     </row>
-    <row r="260" spans="1:10">
+    <row r="260" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A260">
         <v>111</v>
       </c>
@@ -12927,7 +12930,7 @@
         <v>1357</v>
       </c>
     </row>
-    <row r="261" spans="1:10">
+    <row r="261" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A261">
         <v>81</v>
       </c>
@@ -12959,7 +12962,7 @@
         <v>1361</v>
       </c>
     </row>
-    <row r="262" spans="1:10">
+    <row r="262" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A262">
         <v>135</v>
       </c>
@@ -12991,7 +12994,7 @@
         <v>1365</v>
       </c>
     </row>
-    <row r="263" spans="1:10">
+    <row r="263" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A263">
         <v>167</v>
       </c>
@@ -13023,7 +13026,7 @@
         <v>1367</v>
       </c>
     </row>
-    <row r="264" spans="1:10">
+    <row r="264" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A264">
         <v>82</v>
       </c>
@@ -13055,7 +13058,7 @@
         <v>1369</v>
       </c>
     </row>
-    <row r="265" spans="1:10">
+    <row r="265" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A265">
         <v>268</v>
       </c>
@@ -13087,7 +13090,7 @@
         <v>1376</v>
       </c>
     </row>
-    <row r="266" spans="1:10">
+    <row r="266" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A266">
         <v>234</v>
       </c>
@@ -13119,7 +13122,7 @@
         <v>1379</v>
       </c>
     </row>
-    <row r="267" spans="1:10">
+    <row r="267" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A267">
         <v>93</v>
       </c>
@@ -13151,7 +13154,7 @@
         <v>1381</v>
       </c>
     </row>
-    <row r="268" spans="1:10">
+    <row r="268" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A268">
         <v>61</v>
       </c>
@@ -13183,7 +13186,7 @@
         <v>1383</v>
       </c>
     </row>
-    <row r="269" spans="1:10">
+    <row r="269" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A269">
         <v>88</v>
       </c>
@@ -13215,7 +13218,7 @@
         <v>1385</v>
       </c>
     </row>
-    <row r="270" spans="1:10">
+    <row r="270" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A270">
         <v>67</v>
       </c>
@@ -13247,7 +13250,7 @@
         <v>1389</v>
       </c>
     </row>
-    <row r="271" spans="1:10">
+    <row r="271" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A271">
         <v>84</v>
       </c>
@@ -13279,7 +13282,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="272" spans="1:10">
+    <row r="272" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A272">
         <v>20</v>
       </c>
@@ -13311,7 +13314,7 @@
         <v>1399</v>
       </c>
     </row>
-    <row r="273" spans="1:10">
+    <row r="273" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A273">
         <v>25</v>
       </c>
@@ -13344,6 +13347,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A2:J273" xr:uid="{56E4E094-9D27-4105-A489-8372C22533B2}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:J273">
     <sortCondition ref="B3:B273"/>
   </sortState>
@@ -13352,6 +13356,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D1A8D01A0FF9634DB9EFCC8DB434C250" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c80a4892fb4f71f32cde23d159eac728">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f6c6ccbd-788d-45f7-ad1a-adfb240cb0a6" xmlns:ns3="4f8930c7-6a4d-4434-ac67-2594913ad2f7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="83628a1c4b7e3c348e7a2dad63356239" ns2:_="" ns3:_="">
     <xsd:import namespace="f6c6ccbd-788d-45f7-ad1a-adfb240cb0a6"/>
@@ -13558,15 +13571,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -13579,13 +13583,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C31B0769-C736-43F8-AFD6-739B5AACD8BC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FDAE2DE-872B-4A7E-B3CA-5F3DEAD8B9DF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FDAE2DE-872B-4A7E-B3CA-5F3DEAD8B9DF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C31B0769-C736-43F8-AFD6-739B5AACD8BC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="f6c6ccbd-788d-45f7-ad1a-adfb240cb0a6"/>
+    <ds:schemaRef ds:uri="4f8930c7-6a4d-4434-ac67-2594913ad2f7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0941D4C5-F74A-4C3B-AE6E-83EC35BD2E93}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0941D4C5-F74A-4C3B-AE6E-83EC35BD2E93}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4f8930c7-6a4d-4434-ac67-2594913ad2f7"/>
+    <ds:schemaRef ds:uri="f6c6ccbd-788d-45f7-ad1a-adfb240cb0a6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>